<commit_message>
Fix StatsCard value text wrapping mid-number
The value font-size used vw (viewport-width) units, but this grid is
auto-fit: growing the window adds more columns instead of widening
each card, so vw badly overestimated the available space and forced
an oversized font that then had to wrap - and overflowWrap:"anywhere"
let it break in the ugliest possible place, mid-digit-group
("6,460" / "000,"). Switches to container query units (cqi), which
scale off the card's own width instead of the viewport, and restricts
wrapping to natural word breaks (the space before the currency unit)
so a number that must wrap still stays intact on one line.
</commit_message>
<xml_diff>
--- a/backend/vetrix_invoices.xlsx
+++ b/backend/vetrix_invoices.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="فاکتورها" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'فاکتورها'!$A$1:$M$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +27,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +57,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,121 +433,297 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>شماره</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>تاریخ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>نوع</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>طرف‌حساب</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>جمع جزء</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>تخفیف</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>مالیات</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>حمل</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>مبلغ نهایی</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>تسویه‌شده</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>باقی‌مانده</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>وضعیت</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ارز</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17 21:32:44</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>buy</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>سعید</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>final</t>
+      <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:36:12</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>سینا</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>20000</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>final</t>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 06:57:41</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>سینا</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>40000</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>final</t>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:53:03</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>سعید</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>600000</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>final</t>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>